<commit_message>
completed the PII extraction, Analysis and  created data for analysis
</commit_message>
<xml_diff>
--- a/chat_analysis_clean.xlsx
+++ b/chat_analysis_clean.xlsx
@@ -569,7 +569,7 @@
       <c r="H2" t="inlineStr"/>
       <c r="I2" t="inlineStr">
         <is>
-          <t>ORD-445621, Order number</t>
+          <t>Order number, ORD-445621</t>
         </is>
       </c>
       <c r="J2" t="inlineStr"/>
@@ -668,11 +668,7 @@
           <t>Got it. May I know the reason for cancellation?</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>switching providers</t>
-        </is>
-      </c>
+      <c r="F4" t="inlineStr"/>
       <c r="G4" t="inlineStr">
         <is>
           <t>sarah.johnson@live.com</t>
@@ -1311,7 +1307,7 @@
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>order shipped, ORD-112233-X</t>
+          <t>ORD-112233-X, order shipped</t>
         </is>
       </c>
       <c r="J15" t="inlineStr"/>

</xml_diff>